<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-25 15:36 UTC
</commit_message>
<xml_diff>
--- a/data/50001514 - CLIENTE POR DEFINIR A.xlsx
+++ b/data/50001514 - CLIENTE POR DEFINIR A.xlsx
@@ -1826,9 +1826,11 @@
       <c r="B10" s="5">
         <v>46064.97598212963</v>
       </c>
-      <c r="C10" s="6"/>
+      <c r="C10" s="5">
+        <v>46198.63353439815</v>
+      </c>
       <c r="D10" s="5">
-        <v>46196.784762916664</v>
+        <v>46198.633536724534</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>45</v>
@@ -5181,9 +5183,11 @@
       <c r="B65" s="8">
         <v>46064.97597479167</v>
       </c>
-      <c r="C65" s="9"/>
+      <c r="C65" s="8">
+        <v>46198.63385663195</v>
+      </c>
       <c r="D65" s="8">
-        <v>46197.71022986111</v>
+        <v>46198.63385799769</v>
       </c>
       <c r="E65" s="9" t="s">
         <v>234</v>
@@ -5232,7 +5236,7 @@
         <v>46197.5838743287</v>
       </c>
       <c r="D66" s="5">
-        <v>46197.583876261575</v>
+        <v>46198.63395618055</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>237</v>
@@ -5275,7 +5279,7 @@
         <v>46135</v>
       </c>
       <c r="S66" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T66" s="10" t="s">
         <v>31</v>
@@ -5295,7 +5299,7 @@
         <v>46197.71009467593</v>
       </c>
       <c r="D67" s="8">
-        <v>46197.71009662037</v>
+        <v>46198.63395686343</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>243</v>
@@ -5338,7 +5342,7 @@
         <v>46136</v>
       </c>
       <c r="S67" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T67" s="10" t="s">
         <v>31</v>
@@ -5358,7 +5362,7 @@
         <v>46197.71018288194</v>
       </c>
       <c r="D68" s="5">
-        <v>46197.71018483797</v>
+        <v>46198.633957453705</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>247</v>
@@ -5401,7 +5405,7 @@
         <v>46139</v>
       </c>
       <c r="S68" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T68" s="12" t="s">
         <v>249</v>
@@ -5421,7 +5425,7 @@
         <v>46197.71022226852</v>
       </c>
       <c r="D69" s="8">
-        <v>46197.71049135417</v>
+        <v>46198.63395809028</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>251</v>
@@ -5464,7 +5468,7 @@
         <v>46140</v>
       </c>
       <c r="S69" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T69" s="12" t="s">
         <v>249</v>
@@ -5653,9 +5657,11 @@
       <c r="B73" s="8">
         <v>46090.53176077546</v>
       </c>
-      <c r="C73" s="9"/>
+      <c r="C73" s="8">
+        <v>46198.63384538195</v>
+      </c>
       <c r="D73" s="8">
-        <v>46126.792140405094</v>
+        <v>46198.63384679398</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>264</v>
@@ -5700,9 +5706,11 @@
       <c r="B74" s="5">
         <v>46090.53365568287</v>
       </c>
-      <c r="C74" s="6"/>
+      <c r="C74" s="5">
+        <v>46198.63364987269</v>
+      </c>
       <c r="D74" s="5">
-        <v>46197.71023440972</v>
+        <v>46198.633871805556</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>267</v>
@@ -5747,7 +5755,7 @@
         <v>46141</v>
       </c>
       <c r="S74" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T74" s="11" t="s">
         <v>115</v>
@@ -5763,9 +5771,11 @@
       <c r="B75" s="8">
         <v>46090.53385733796</v>
       </c>
-      <c r="C75" s="9"/>
+      <c r="C75" s="8">
+        <v>46198.63376841435</v>
+      </c>
       <c r="D75" s="8">
-        <v>46161.167864664356</v>
+        <v>46198.63389696759</v>
       </c>
       <c r="E75" s="9" t="s">
         <v>270</v>
@@ -5810,7 +5820,7 @@
         <v>46153</v>
       </c>
       <c r="S75" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T75" s="11" t="s">
         <v>115</v>

</xml_diff>

<commit_message>
Curva S actualizada 2026-07-10 17:20 Chile
</commit_message>
<xml_diff>
--- a/data/50001514 - CLIENTE POR DEFINIR A.xlsx
+++ b/data/50001514 - CLIENTE POR DEFINIR A.xlsx
@@ -5486,7 +5486,7 @@
       </c>
       <c r="C70" s="6"/>
       <c r="D70" s="5">
-        <v>46126.792140254634</v>
+        <v>46213.83018092593</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>254</v>
@@ -5531,9 +5531,11 @@
       <c r="B71" s="8">
         <v>46064.97597436343</v>
       </c>
-      <c r="C71" s="9"/>
+      <c r="C71" s="8">
+        <v>46213.83015892361</v>
+      </c>
       <c r="D71" s="8">
-        <v>46197.71023167824</v>
+        <v>46213.830161307866</v>
       </c>
       <c r="E71" s="9" t="s">
         <v>257</v>
@@ -5594,9 +5596,11 @@
       <c r="B72" s="5">
         <v>46064.975974050925</v>
       </c>
-      <c r="C72" s="6"/>
+      <c r="C72" s="5">
+        <v>46213.83017385416</v>
+      </c>
       <c r="D72" s="5">
-        <v>46197.710233125</v>
+        <v>46213.83017636574</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>261</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-21 15:08 UTC
</commit_message>
<xml_diff>
--- a/data/50001514 - CLIENTE POR DEFINIR A.xlsx
+++ b/data/50001514 - CLIENTE POR DEFINIR A.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="916" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="917" uniqueCount="269">
   <si>
     <t>50001514 - CLIENTE POR DEFINIR</t>
   </si>
@@ -4992,7 +4992,7 @@
         <v>46107.71404958333</v>
       </c>
       <c r="D62" s="5">
-        <v>46139.78118356482</v>
+        <v>46224.574943750005</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>223</v>
@@ -5001,9 +5001,11 @@
         <v>26</v>
       </c>
       <c r="G62" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H62" s="6"/>
+        <v>88</v>
+      </c>
+      <c r="H62" s="6" t="s">
+        <v>88</v>
+      </c>
       <c r="I62" s="6"/>
       <c r="J62" s="5">
         <v>46122</v>

</xml_diff>